<commit_message>
Naming of variables to match SweFor d:o. Error correction in comd. Adding variable DeadWood.
</commit_message>
<xml_diff>
--- a/GayaSpecs2603.xlsx
+++ b/GayaSpecs2603.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jola\Dropbox\Jola\Applications\GAYA\G3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jola\source\repos\LjuskOlaEriksson\GAYA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B5ACAD-1BCC-4DA5-B5FF-D54C9AD7BCD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25B4357-885E-4E28-BACA-41D788C92CDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3084" yWindow="2520" windowWidth="17280" windowHeight="9960" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Example" sheetId="4" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="417">
   <si>
     <t>LOG</t>
   </si>
@@ -740,9 +740,6 @@
     <t>Dynamic variables</t>
   </si>
   <si>
-    <t>Static variables</t>
-  </si>
-  <si>
     <t>Number of stems (/ha)</t>
   </si>
   <si>
@@ -1238,9 +1235,6 @@
     <t>number of stems for species 1-12</t>
   </si>
   <si>
-    <t>4-16</t>
-  </si>
-  <si>
     <t>17-28</t>
   </si>
   <si>
@@ -1281,6 +1275,18 @@
   </si>
   <si>
     <t>FFOREST C:/.../SegmentData_Big.csv</t>
+  </si>
+  <si>
+    <t>total age or time since final harvest</t>
+  </si>
+  <si>
+    <t>5-16</t>
+  </si>
+  <si>
+    <t>Static variables (integers)</t>
+  </si>
+  <si>
+    <t>Static variables (real)</t>
   </si>
 </sst>
 </file>
@@ -1731,7 +1737,7 @@
   <sheetData>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1739,23 +1745,23 @@
         <v>0</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1768,18 +1774,18 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1789,23 +1795,23 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -1813,15 +1819,15 @@
         <v>126</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -1829,7 +1835,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -1837,92 +1843,92 @@
         <v>6</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
@@ -1932,58 +1938,58 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -1996,23 +2002,23 @@
         <v>126</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -2035,138 +2041,138 @@
         <v>151</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
@@ -2174,12 +2180,12 @@
         <v>3</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
@@ -2189,7 +2195,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
@@ -2252,7 +2258,7 @@
         <v>31</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -2276,7 +2282,7 @@
         <v>69</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -2290,7 +2296,7 @@
         <v>160</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -2301,12 +2307,12 @@
         <v>39</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="P11" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -2317,7 +2323,7 @@
         <v>34</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
@@ -2328,7 +2334,7 @@
         <v>94</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -2339,7 +2345,7 @@
         <v>95</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
@@ -2369,7 +2375,7 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C17" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>74</v>
@@ -2383,10 +2389,10 @@
         <v>97</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
@@ -2394,12 +2400,12 @@
         <v>22</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
@@ -2407,7 +2413,7 @@
         <v>35</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
@@ -2415,15 +2421,15 @@
         <v>36</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>292</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
@@ -2456,7 +2462,7 @@
         <v>35</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
@@ -2464,7 +2470,7 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
@@ -2485,26 +2491,26 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -2512,12 +2518,12 @@
         <v>35</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -2980,7 +2986,7 @@
         <v>18</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2993,12 +2999,12 @@
         <v>35</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B107" s="1" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>201</v>
@@ -3014,7 +3020,7 @@
         <v>44</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.25">
@@ -3056,20 +3062,20 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C115" s="1" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C116" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.25">
@@ -3084,7 +3090,7 @@
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C121" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.25">
@@ -3397,19 +3403,18 @@
     <col min="7" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B1" s="2"/>
       <c r="C1" s="1" t="s">
-        <v>234</v>
+        <v>415</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1" ht="26.4" x14ac:dyDescent="0.25">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>203</v>
       </c>
@@ -3420,16 +3425,16 @@
         <v>205</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>204</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>75</v>
       </c>
@@ -3440,16 +3445,16 @@
         <v>173</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>206</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>76</v>
       </c>
@@ -3460,16 +3465,16 @@
         <v>208</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>45</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>77</v>
       </c>
@@ -3480,58 +3485,58 @@
         <v>210</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>209</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>207</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>212</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>213</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>215</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>78</v>
       </c>
@@ -3542,10 +3547,10 @@
         <v>217</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>214</v>
       </c>
@@ -3556,151 +3561,151 @@
         <v>219</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>216</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>218</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>220</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>221</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>222</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>223</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>224</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>225</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>226</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>228</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>229</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>230</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>231</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>232</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>
@@ -3711,7 +3716,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CCBC7E8-6034-45A9-83C3-EBFCC230AE01}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="8.88671875" style="1"/>
@@ -3719,36 +3724,36 @@
   <sheetData>
     <row r="1" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>390</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>391</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3756,10 +3761,10 @@
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>393</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -3767,10 +3772,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>395</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -3778,85 +3783,96 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>4</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>397</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>400</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>399</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>401</v>
+        <v>414</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>402</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>406</v>
-      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>409</v>
+      <c r="A14" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>407</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6"/>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>